<commit_message>
feat(divergent-universe): G11-P3-B6 verify Sora release artifacts
</commit_message>
<xml_diff>
--- a/config/divergent-universe-generated/templates/DivergentUniverse.xlsx
+++ b/config/divergent-universe-generated/templates/DivergentUniverse.xlsx
@@ -100,7 +100,7 @@
     <t>@schema</t>
   </si>
   <si>
-    <t>a1e609ab589cf10f</t>
+    <t>87e82545945935af</t>
   </si>
   <si>
     <t>#name</t>
@@ -172,13 +172,13 @@
     <t>string</t>
   </si>
   <si>
-    <t>enum&lt;DUOwnership&gt;</t>
-  </si>
-  <si>
-    <t>enum&lt;DUCoverageState&gt;</t>
-  </si>
-  <si>
-    <t>enum&lt;DUEvidenceQuality&gt;</t>
+    <t>enum&lt;DuOwnership&gt;</t>
+  </si>
+  <si>
+    <t>enum&lt;DuCoverageState&gt;</t>
+  </si>
+  <si>
+    <t>enum&lt;DuEvidenceQuality&gt;</t>
   </si>
   <si>
     <t>optional&lt;list&lt;ref&lt;DivergentUniverseSources.id&gt;&gt;&gt;</t>
@@ -235,7 +235,7 @@
     <t>DivergentUniverseModules</t>
   </si>
   <si>
-    <t>9afad6debafd732e</t>
+    <t>5a18d35a75bf680e</t>
   </si>
   <si>
     <t>sub_mode</t>
@@ -253,7 +253,7 @@
     <t>DivergentUniverseEntries</t>
   </si>
   <si>
-    <t>e0bb186de85bc31f</t>
+    <t>bc5fde22f56064bf</t>
   </si>
   <si>
     <t>entry_kind</t>
@@ -265,7 +265,7 @@
     <t>DivergentUniverseFinishConditions</t>
   </si>
   <si>
-    <t>8839250898cdcbe5</t>
+    <t>784f78fb4e12fb05</t>
   </si>
   <si>
     <t>condition_kind</t>
@@ -280,7 +280,7 @@
     <t>DivergentUniverseAreas</t>
   </si>
   <si>
-    <t>0b01f13e373549e6</t>
+    <t>38f7ba402c6f1946</t>
   </si>
   <si>
     <t>difficulty_ids</t>
@@ -304,7 +304,7 @@
     <t>DivergentUniverseDifficulties</t>
   </si>
   <si>
-    <t>8e75e03f2cc31fd3</t>
+    <t>9190266d8ad95c33</t>
   </si>
   <si>
     <t>level_list</t>
@@ -319,7 +319,7 @@
     <t>DivergentUniverseLayers</t>
   </si>
   <si>
-    <t>e73aec14509cf8f5</t>
+    <t>d7bd0e8c8d275115</t>
   </si>
   <si>
     <t>layer_number</t>
@@ -331,7 +331,7 @@
     <t>DivergentUniverseLayerRooms</t>
   </si>
   <si>
-    <t>ca398e3e080bd2cd</t>
+    <t>055c66c8f465f76d</t>
   </si>
   <si>
     <t>layer_id</t>
@@ -349,7 +349,7 @@
     <t>DivergentUniverseRooms</t>
   </si>
   <si>
-    <t>cbba855fcc8cbfdc</t>
+    <t>5aac27c2d16d723c</t>
   </si>
   <si>
     <t>room_type</t>
@@ -364,7 +364,7 @@
     <t>DivergentUniverseStageFlow</t>
   </si>
   <si>
-    <t>85bd7b88adbb187d</t>
+    <t>b421d44bb4eb829d</t>
   </si>
   <si>
     <t>entry_id</t>
@@ -382,7 +382,7 @@
     <t>DivergentUniverseCyclicalChallenges</t>
   </si>
   <si>
-    <t>292aad3753e0cc29</t>
+    <t>7c426538bf1cd2c9</t>
   </si>
   <si>
     <t>area_id</t>
@@ -403,7 +403,7 @@
     <t>DivergentUniverseProtocols</t>
   </si>
   <si>
-    <t>a790c644775ea6c5</t>
+    <t>593a1e5ac5317de5</t>
   </si>
   <si>
     <t>protocol_level</t>
@@ -421,7 +421,7 @@
     <t>DivergentUniverseAstronomicalDivisions</t>
   </si>
   <si>
-    <t>d3414782f5beb9a2</t>
+    <t>e96c2579e6252c42</t>
   </si>
   <si>
     <t>division_level</t>
@@ -436,7 +436,7 @@
     <t>DivergentUniverseStarPioneerPractice</t>
   </si>
   <si>
-    <t>e25aa96ed3365311</t>
+    <t>11c47b469312c131</t>
   </si>
   <si>
     <t>mode_kind</t>
@@ -448,7 +448,7 @@
     <t>DivergentUniverseCognoculi</t>
   </si>
   <si>
-    <t>0420468b75b0f65e</t>
+    <t>6942c546e656c57e</t>
   </si>
   <si>
     <t>source_locator</t>
@@ -463,7 +463,7 @@
     <t>DivergentUniverseArithmeticMappingEligibility</t>
   </si>
   <si>
-    <t>f04cce7fb3171d5b</t>
+    <t>20b8a6b6ab3d347b</t>
   </si>
   <si>
     <t>avatar_id</t>
@@ -478,7 +478,7 @@
     <t>DivergentUniverseArithmeticMappingBuilds</t>
   </si>
   <si>
-    <t>1249dfc52e68c923</t>
+    <t>ecc3c87378bd6a43</t>
   </si>
   <si>
     <t>level</t>
@@ -499,7 +499,7 @@
     <t>DivergentUniverseArithmeticMappingRules</t>
   </si>
   <si>
-    <t>3d71a0826f22e288</t>
+    <t>beb0cd1360417f68</t>
   </si>
   <si>
     <t>selection_timing</t>
@@ -517,7 +517,7 @@
     <t>DivergentUniverseEquations</t>
   </si>
   <si>
-    <t>2c09347543c22879</t>
+    <t>6f37548f1bce71d9</t>
   </si>
   <si>
     <t>recipe_id</t>
@@ -541,7 +541,7 @@
     <t>DivergentUniverseEquationRecipes</t>
   </si>
   <si>
-    <t>ebc94c403de2e0cb</t>
+    <t>ffccd420ad25256b</t>
   </si>
   <si>
     <t>equation_id</t>
@@ -562,7 +562,7 @@
     <t>DivergentUniverseEquationCategories</t>
   </si>
   <si>
-    <t>a1a2b9dc0ec93478</t>
+    <t>40bba903f15e4798</t>
   </si>
   <si>
     <t>offer_rules</t>
@@ -574,7 +574,7 @@
     <t>DivergentUniverseEquationOffers</t>
   </si>
   <si>
-    <t>ecc1101ecbe4684b</t>
+    <t>2b7a5639135c3eab</t>
   </si>
   <si>
     <t>candidate_ids</t>
@@ -592,7 +592,7 @@
     <t>DivergentUniverseEquationProgress</t>
   </si>
   <si>
-    <t>1959610613ad444e</t>
+    <t>d782c6c83713c22e</t>
   </si>
   <si>
     <t>contribution_rule</t>
@@ -604,7 +604,7 @@
     <t>DivergentUniverseEquationExpansionStates</t>
   </si>
   <si>
-    <t>68dc817aee17d43b</t>
+    <t>b67a095200ff9f5b</t>
   </si>
   <si>
     <t>state</t>
@@ -619,7 +619,7 @@
     <t>DivergentUniverseEquationEffects</t>
   </si>
   <si>
-    <t>d95757708f45d620</t>
+    <t>95a9a61be6942680</t>
   </si>
   <si>
     <t>keyword_ids</t>
@@ -631,7 +631,7 @@
     <t>DivergentUniverseEquationReplacementRules</t>
   </si>
   <si>
-    <t>330a9638d5e07d16</t>
+    <t>87b69c662e60a876</t>
   </si>
   <si>
     <t>operation</t>
@@ -646,7 +646,7 @@
     <t>DivergentUniverseBlessingPaths</t>
   </si>
   <si>
-    <t>bc1526088c981784</t>
+    <t>e722d7554fac0fe4</t>
   </si>
   <si>
     <t>path_id</t>
@@ -661,7 +661,7 @@
     <t>DivergentUniverseBlessings</t>
   </si>
   <si>
-    <t>18a40f3980c9126a</t>
+    <t>3f7f44268d16154a</t>
   </si>
   <si>
     <t>level_ids</t>
@@ -670,7 +670,7 @@
     <t>DivergentUniverseBlessingLevels</t>
   </si>
   <si>
-    <t>48dc238357e3dda7</t>
+    <t>20ea69f4e8d43107</t>
   </si>
   <si>
     <t>blessing_id</t>
@@ -682,7 +682,7 @@
     <t>DivergentUniverseBlessingGroups</t>
   </si>
   <si>
-    <t>339142cd75d8e85f</t>
+    <t>08c18ff88964ceff</t>
   </si>
   <si>
     <t>selection_policy</t>
@@ -691,7 +691,7 @@
     <t>DivergentUniverseBlessingRewriteRules</t>
   </si>
   <si>
-    <t>ada10de46e3f26d0</t>
+    <t>83836f6870d09830</t>
   </si>
   <si>
     <t>input_blessing_id</t>
@@ -712,7 +712,7 @@
     <t>DivergentUniverseBlessingEquationContributions</t>
   </si>
   <si>
-    <t>156746ad46980e75</t>
+    <t>37ff39692102e015</t>
   </si>
   <si>
     <t>equation_ids</t>
@@ -727,7 +727,7 @@
     <t>DivergentUniverseCurios</t>
   </si>
   <si>
-    <t>886c0f9d7fcb71c4</t>
+    <t>75c158400c465264</t>
   </si>
   <si>
     <t>state_ids</t>
@@ -739,7 +739,7 @@
     <t>DivergentUniverseCurioStates</t>
   </si>
   <si>
-    <t>deb96f83e79a111f</t>
+    <t>53004453d83392ff</t>
   </si>
   <si>
     <t>curio_id</t>
@@ -754,7 +754,7 @@
     <t>DivergentUniverseCurioGroups</t>
   </si>
   <si>
-    <t>7d4b8ca41332264c</t>
+    <t>91b996eba7358d2c</t>
   </si>
   <si>
     <t>candidate_state_ids</t>
@@ -766,7 +766,7 @@
     <t>DivergentUniverseCurioLifecycleRules</t>
   </si>
   <si>
-    <t>0cb116c2d162c37b</t>
+    <t>f364887b6eff481b</t>
   </si>
   <si>
     <t>activation</t>
@@ -784,7 +784,7 @@
     <t>DivergentUniverseGrandMiracles</t>
   </si>
   <si>
-    <t>f3967d3357eb2b45</t>
+    <t>cc363dd44f5c3ba5</t>
   </si>
   <si>
     <t>display_id</t>
@@ -796,7 +796,7 @@
     <t>DivergentUniverseGrandMiracleEligibility</t>
   </si>
   <si>
-    <t>3dca4b272e762e96</t>
+    <t>ec837451d97f2db6</t>
   </si>
   <si>
     <t>grand_miracle_id</t>
@@ -814,7 +814,7 @@
     <t>DivergentUniverseGrandMiracleStates</t>
   </si>
   <si>
-    <t>2951c92b43baef94</t>
+    <t>18d8c21789a553f4</t>
   </si>
   <si>
     <t>duration</t>
@@ -823,7 +823,7 @@
     <t>DivergentUniverseTitanTypes</t>
   </si>
   <si>
-    <t>ec5203f4045a9aad</t>
+    <t>10d8f2a9c89af50d</t>
   </si>
   <si>
     <t>boon_ids</t>
@@ -835,7 +835,7 @@
     <t>DivergentUniverseTitanBoons</t>
   </si>
   <si>
-    <t>3cd15874333d5317</t>
+    <t>8ee36e31d71c0a37</t>
   </si>
   <si>
     <t>titan_type</t>
@@ -853,7 +853,7 @@
     <t>DivergentUniverseTitanTalents</t>
   </si>
   <si>
-    <t>32e92a244d57de7f</t>
+    <t>4812097243aded9f</t>
   </si>
   <si>
     <t>cost</t>
@@ -865,7 +865,7 @@
     <t>DivergentUniverseTitanChoices</t>
   </si>
   <si>
-    <t>448e3381c6062986</t>
+    <t>a91949959fabe8e6</t>
   </si>
   <si>
     <t>selection_count</t>
@@ -877,7 +877,7 @@
     <t>DivergentUniverseTitanContributions</t>
   </si>
   <si>
-    <t>f86f219c3feb4309</t>
+    <t>35818620cb58cae9</t>
   </si>
   <si>
     <t>scope</t>
@@ -889,7 +889,7 @@
     <t>DivergentUniverseWorkbenches</t>
   </si>
   <si>
-    <t>72ccd840ae199f64</t>
+    <t>cfbc81d3a477a7c4</t>
   </si>
   <si>
     <t>function_ids</t>
@@ -910,7 +910,7 @@
     <t>DivergentUniverseWorkbenchFunctions</t>
   </si>
   <si>
-    <t>6c2003b3a1246bce</t>
+    <t>d5467b80cc73442e</t>
   </si>
   <si>
     <t>function_type</t>
@@ -928,7 +928,7 @@
     <t>DivergentUniverseGambleGroups</t>
   </si>
   <si>
-    <t>b6106f8614a1222c</t>
+    <t>83d42c148e44eb8c</t>
   </si>
   <si>
     <t>group_type</t>
@@ -943,7 +943,7 @@
     <t>DivergentUniverseGambleUnits</t>
   </si>
   <si>
-    <t>2ecdd83cd5a8af05</t>
+    <t>5f8ceb1d686859a5</t>
   </si>
   <si>
     <t>unit_type</t>
@@ -955,7 +955,7 @@
     <t>DivergentUniverseCurseChests</t>
   </si>
   <si>
-    <t>3855d43f0c8a2596</t>
+    <t>0dac35d4ad1d4df6</t>
   </si>
   <si>
     <t>chest_type</t>
@@ -967,7 +967,7 @@
     <t>DivergentUniverseCurrencies</t>
   </si>
   <si>
-    <t>831c8916d30952b6</t>
+    <t>452182101bdb41d6</t>
   </si>
   <si>
     <t>gain_rules</t>
@@ -982,7 +982,7 @@
     <t>DivergentUniverseServiceRules</t>
   </si>
   <si>
-    <t>3c746d474228c4a7</t>
+    <t>3c3543ffd2c70547</t>
   </si>
   <si>
     <t>currency_id</t>
@@ -1003,7 +1003,7 @@
     <t>DivergentUniverseServiceOfferRules</t>
   </si>
   <si>
-    <t>575ede7ecd84be5a</t>
+    <t>a1ec343fcf33dfba</t>
   </si>
   <si>
     <t>service_id</t>
@@ -1015,7 +1015,7 @@
     <t>DivergentUniversePermanentTalents</t>
   </si>
   <si>
-    <t>2c6d79a830b5605b</t>
+    <t>7188e173c94e0e7b</t>
   </si>
   <si>
     <t>prerequisite_ids</t>
@@ -1030,7 +1030,7 @@
     <t>DivergentUniverseUnlocks</t>
   </si>
   <si>
-    <t>8541b3be8a239c91</t>
+    <t>fcea47d7ceda2571</t>
   </si>
   <si>
     <t>finish_condition_id</t>
@@ -1045,7 +1045,7 @@
     <t>DivergentUniverseCommonConstants</t>
   </si>
   <si>
-    <t>a3088ee8fe55710f</t>
+    <t>83366f9c5d4d886f</t>
   </si>
   <si>
     <t>value_kind</t>
@@ -1060,7 +1060,7 @@
     <t>DivergentUniverseWeeklyModifiers</t>
   </si>
   <si>
-    <t>3d127585956d0eba</t>
+    <t>8516ccfa5d76719a</t>
   </si>
   <si>
     <t>content_ids</t>
@@ -1075,7 +1075,7 @@
     <t>DivergentUniverseRoomMarks</t>
   </si>
   <si>
-    <t>42917e47f4ae03b4</t>
+    <t>d29c4eb81adeadd4</t>
   </si>
   <si>
     <t>mark_kind</t>
@@ -1087,7 +1087,7 @@
     <t>DivergentUniverseProgressionEffects</t>
   </si>
   <si>
-    <t>3d409b3a28bb0491</t>
+    <t>db79ceddcfbf31b1</t>
   </si>
 </sst>
 </file>
@@ -1883,14 +1883,14 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DUOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
       <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DUCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DUEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
-      <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, ExactOfficialText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DuEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+      <formula1>"ExactStructured,ExactPublicText,ExactOfficialText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2274,14 +2274,14 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DUOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
       <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DUCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DUEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
-      <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, ExactOfficialText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DuEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+      <formula1>"ExactStructured,ExactPublicText,ExactOfficialText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2666,14 +2666,14 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DUOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
       <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DUCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DUEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
-      <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, ExactOfficialText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DuEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+      <formula1>"ExactStructured,ExactPublicText,ExactOfficialText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3057,14 +3057,14 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DUOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
       <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DUCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DUEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
-      <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, ExactOfficialText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DuEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+      <formula1>"ExactStructured,ExactPublicText,ExactOfficialText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3434,14 +3434,14 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DUOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
       <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DUCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DUEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
-      <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, ExactOfficialText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DuEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+      <formula1>"ExactStructured,ExactPublicText,ExactOfficialText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3825,14 +3825,14 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DUOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
       <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DUCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DUEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
-      <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, ExactOfficialText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DuEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+      <formula1>"ExactStructured,ExactPublicText,ExactOfficialText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4200,14 +4200,14 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DUOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
       <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DUCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DUEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
-      <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, ExactOfficialText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DuEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+      <formula1>"ExactStructured,ExactPublicText,ExactOfficialText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4576,14 +4576,14 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DUOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
       <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DUCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DUEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
-      <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, ExactOfficialText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DuEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+      <formula1>"ExactStructured,ExactPublicText,ExactOfficialText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4993,14 +4993,14 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DUOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
       <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DUCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DUEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
-      <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, ExactOfficialText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DuEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+      <formula1>"ExactStructured,ExactPublicText,ExactOfficialText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5384,14 +5384,14 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DUOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
       <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DUCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DUEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
-      <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, ExactOfficialText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DuEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+      <formula1>"ExactStructured,ExactPublicText,ExactOfficialText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5791,14 +5791,14 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DUOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
       <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DUCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DUEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
-      <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, ExactOfficialText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DuEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+      <formula1>"ExactStructured,ExactPublicText,ExactOfficialText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6180,14 +6180,14 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DUOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
       <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DUCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DUEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
-      <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, ExactOfficialText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DuEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+      <formula1>"ExactStructured,ExactPublicText,ExactOfficialText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6572,14 +6572,14 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DUOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
       <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DUCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DUEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
-      <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, ExactOfficialText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DuEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+      <formula1>"ExactStructured,ExactPublicText,ExactOfficialText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6948,14 +6948,14 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DUOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
       <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DUCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DUEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
-      <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, ExactOfficialText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DuEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+      <formula1>"ExactStructured,ExactPublicText,ExactOfficialText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -7337,14 +7337,14 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DUOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
       <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DUCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DUEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
-      <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, ExactOfficialText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DuEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+      <formula1>"ExactStructured,ExactPublicText,ExactOfficialText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -7729,14 +7729,14 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DUOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
       <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DUCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DUEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
-      <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, ExactOfficialText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DuEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+      <formula1>"ExactStructured,ExactPublicText,ExactOfficialText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -8120,14 +8120,14 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DUOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
       <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DUCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DUEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
-      <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, ExactOfficialText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DuEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+      <formula1>"ExactStructured,ExactPublicText,ExactOfficialText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -8510,14 +8510,14 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DUOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
       <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DUCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DUEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
-      <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, ExactOfficialText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DuEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+      <formula1>"ExactStructured,ExactPublicText,ExactOfficialText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -8899,14 +8899,14 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DUOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
       <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DUCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DUEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
-      <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, ExactOfficialText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DuEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+      <formula1>"ExactStructured,ExactPublicText,ExactOfficialText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -9274,14 +9274,14 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DUOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
       <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DUCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DUEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
-      <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, ExactOfficialText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DuEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+      <formula1>"ExactStructured,ExactPublicText,ExactOfficialText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -9663,14 +9663,14 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DUOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
       <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DUCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DUEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
-      <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, ExactOfficialText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DuEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+      <formula1>"ExactStructured,ExactPublicText,ExactOfficialText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -10054,14 +10054,14 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DUOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
       <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DUCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DUEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
-      <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, ExactOfficialText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DuEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+      <formula1>"ExactStructured,ExactPublicText,ExactOfficialText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -10431,14 +10431,14 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DUOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
       <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DUCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DUEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
-      <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, ExactOfficialText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DuEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+      <formula1>"ExactStructured,ExactPublicText,ExactOfficialText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -10806,14 +10806,14 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DUOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
       <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DUCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DUEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
-      <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, ExactOfficialText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DuEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+      <formula1>"ExactStructured,ExactPublicText,ExactOfficialText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -11225,14 +11225,14 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DUOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
       <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DUCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DUEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
-      <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, ExactOfficialText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DuEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+      <formula1>"ExactStructured,ExactPublicText,ExactOfficialText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -11632,14 +11632,14 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DUOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
       <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DUCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DUEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
-      <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, ExactOfficialText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DuEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+      <formula1>"ExactStructured,ExactPublicText,ExactOfficialText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -12008,14 +12008,14 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DUOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
       <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DUCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DUEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
-      <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, ExactOfficialText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DuEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+      <formula1>"ExactStructured,ExactPublicText,ExactOfficialText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -12399,14 +12399,14 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DUOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
       <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DUCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DUEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
-      <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, ExactOfficialText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DuEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+      <formula1>"ExactStructured,ExactPublicText,ExactOfficialText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -12776,14 +12776,14 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DUOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
       <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DUCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DUEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
-      <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, ExactOfficialText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DuEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+      <formula1>"ExactStructured,ExactPublicText,ExactOfficialText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -13195,14 +13195,14 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DUOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
       <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DUCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DUEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
-      <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, ExactOfficialText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DuEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+      <formula1>"ExactStructured,ExactPublicText,ExactOfficialText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -13584,14 +13584,14 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DUOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
       <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DUCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DUEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
-      <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, ExactOfficialText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DuEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+      <formula1>"ExactStructured,ExactPublicText,ExactOfficialText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -13975,14 +13975,14 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DUOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
       <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DUCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DUEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
-      <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, ExactOfficialText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DuEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+      <formula1>"ExactStructured,ExactPublicText,ExactOfficialText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -14380,14 +14380,14 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DUOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
       <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DUCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DUEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
-      <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, ExactOfficialText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DuEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+      <formula1>"ExactStructured,ExactPublicText,ExactOfficialText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -14756,14 +14756,14 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DUOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
       <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DUCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DUEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
-      <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, ExactOfficialText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DuEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+      <formula1>"ExactStructured,ExactPublicText,ExactOfficialText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -15131,14 +15131,14 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DUOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
       <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DUCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DUEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
-      <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, ExactOfficialText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DuEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+      <formula1>"ExactStructured,ExactPublicText,ExactOfficialText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -15536,14 +15536,14 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DUOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
       <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DUCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DUEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
-      <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, ExactOfficialText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DuEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+      <formula1>"ExactStructured,ExactPublicText,ExactOfficialText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -15941,14 +15941,14 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DUOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
       <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DUCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DUEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
-      <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, ExactOfficialText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DuEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+      <formula1>"ExactStructured,ExactPublicText,ExactOfficialText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -16348,14 +16348,14 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DUOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
       <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DUCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DUEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
-      <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, ExactOfficialText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DuEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+      <formula1>"ExactStructured,ExactPublicText,ExactOfficialText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -16723,14 +16723,14 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DUOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
       <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DUCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DUEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
-      <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, ExactOfficialText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DuEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+      <formula1>"ExactStructured,ExactPublicText,ExactOfficialText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -17104,14 +17104,14 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DUOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
       <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DUCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DUEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
-      <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, ExactOfficialText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DuEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+      <formula1>"ExactStructured,ExactPublicText,ExactOfficialText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -17493,14 +17493,14 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DUOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
       <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DUCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DUEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
-      <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, ExactOfficialText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DuEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+      <formula1>"ExactStructured,ExactPublicText,ExactOfficialText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -17868,14 +17868,14 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DUOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
       <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DUCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DUEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
-      <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, ExactOfficialText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DuEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+      <formula1>"ExactStructured,ExactPublicText,ExactOfficialText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -18243,14 +18243,14 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DUOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
       <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DUCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DUEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
-      <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, ExactOfficialText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DuEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+      <formula1>"ExactStructured,ExactPublicText,ExactOfficialText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -18618,14 +18618,14 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DUOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
       <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DUCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DUEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
-      <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, ExactOfficialText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DuEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+      <formula1>"ExactStructured,ExactPublicText,ExactOfficialText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -19013,14 +19013,14 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DUOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
       <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DUCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DUEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
-      <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, ExactOfficialText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DuEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+      <formula1>"ExactStructured,ExactPublicText,ExactOfficialText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -19402,14 +19402,14 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DUOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
       <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DUCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DUEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
-      <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, ExactOfficialText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DuEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+      <formula1>"ExactStructured,ExactPublicText,ExactOfficialText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -19809,14 +19809,14 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DUOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
       <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DUCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DUEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
-      <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, ExactOfficialText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DuEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+      <formula1>"ExactStructured,ExactPublicText,ExactOfficialText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -20212,14 +20212,14 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DUOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
       <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DUCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DUEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
-      <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, ExactOfficialText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DuEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+      <formula1>"ExactStructured,ExactPublicText,ExactOfficialText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -20621,14 +20621,14 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DUOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
       <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DUCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DUEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
-      <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, ExactOfficialText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DuEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+      <formula1>"ExactStructured,ExactPublicText,ExactOfficialText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -20999,14 +20999,14 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DUOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
       <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DUCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DUEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
-      <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, ExactOfficialText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DuEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+      <formula1>"ExactStructured,ExactPublicText,ExactOfficialText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -21374,14 +21374,14 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DUOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
       <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DUCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DUEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
-      <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, ExactOfficialText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DuEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+      <formula1>"ExactStructured,ExactPublicText,ExactOfficialText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -21763,14 +21763,14 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DUOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
       <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DUCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DUEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
-      <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, ExactOfficialText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DuEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+      <formula1>"ExactStructured,ExactPublicText,ExactOfficialText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -22138,14 +22138,14 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DUOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
       <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DUCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DUEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
-      <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, ExactOfficialText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DuEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+      <formula1>"ExactStructured,ExactPublicText,ExactOfficialText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -22500,14 +22500,14 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DUOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
       <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DUCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DUEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
-      <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, ExactOfficialText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DuEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+      <formula1>"ExactStructured,ExactPublicText,ExactOfficialText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -22876,14 +22876,14 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DUOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
       <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DUCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DUEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
-      <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, ExactOfficialText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DuEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+      <formula1>"ExactStructured,ExactPublicText,ExactOfficialText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -23238,14 +23238,14 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DUOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
       <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DUCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DUEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
-      <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, ExactOfficialText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DuEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+      <formula1>"ExactStructured,ExactPublicText,ExactOfficialText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -23615,14 +23615,14 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DUOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
       <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DUCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DUEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
-      <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, ExactOfficialText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DuEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+      <formula1>"ExactStructured,ExactPublicText,ExactOfficialText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -23992,14 +23992,14 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DUOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
       <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DUCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DUEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
-      <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, ExactOfficialText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DuEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+      <formula1>"ExactStructured,ExactPublicText,ExactOfficialText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>